<commit_message>
Update permanent excel data
</commit_message>
<xml_diff>
--- a/api/data.xlsx
+++ b/api/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Downloads\0527_3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB97FC4F-19C6-4E93-AA14-5408FC78886C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2815292-6DE2-463E-9692-BD3D4F46CAD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{F06B8FF0-7C61-4A69-AB6C-473C6FF4E06D}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="50">
   <si>
     <t>담당 부서 및 연락처</t>
   </si>
@@ -350,6 +350,323 @@
         <family val="2"/>
       </rPr>
       <t>.</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+      </rPr>
+      <t>주차</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+      </rPr>
+      <t>주차타워는</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+      </rPr>
+      <t>진행사항은</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+      </rPr>
+      <t>어떻게</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+      </rPr>
+      <t>되나요</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>?</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+      </rPr>
+      <t>주차타워는</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+      </rPr>
+      <t>정문동과</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+      </rPr>
+      <t>연계하여</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+      </rPr>
+      <t>진행되며</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+      </rPr>
+      <t>정확한</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+      </rPr>
+      <t>일정이</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+      </rPr>
+      <t>나오면</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+      </rPr>
+      <t>재공지해</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+      </rPr>
+      <t>드리도록</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+      </rPr>
+      <t>하겠습니다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>.</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+      </rPr>
+      <t>인프라</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+      </rPr>
+      <t>파트</t>
     </r>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -358,7 +675,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -394,8 +711,15 @@
       <family val="3"/>
       <charset val="129"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -408,8 +732,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -418,22 +748,17 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="medium">
-        <color rgb="FF000000"/>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
       </right>
-      <top/>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
@@ -443,24 +768,27 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" readingOrder="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" readingOrder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -776,7 +1104,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45A1DB66-6E91-4520-A1EE-7F17440E0461}">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="10.3984375" bestFit="1" customWidth="1"/>
@@ -785,187 +1113,237 @@
     <col min="4" max="4" width="25.3984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="18" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="18" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" s="3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="18" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D4" s="3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="18" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D5" s="3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="18" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="5" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="18" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="D7" s="3" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="18" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="D8" s="3" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="18" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="D9" s="3" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="18" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="1" t="s">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="D10" s="3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="18" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="D11" s="3" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="18" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="D12" s="1" t="s">
+      <c r="D12" s="3" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="18" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="1" t="s">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C13" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="D13" s="1" t="s">
+      <c r="D13" s="3" t="s">
         <v>40</v>
       </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A15" s="6"/>
+      <c r="B15" s="6"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="6"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A16" s="6"/>
+      <c r="B16" s="6"/>
+      <c r="C16" s="6"/>
+      <c r="D16" s="6"/>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A17" s="6"/>
+      <c r="B17" s="6"/>
+      <c r="C17" s="6"/>
+      <c r="D17" s="6"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A18" s="6"/>
+      <c r="B18" s="6"/>
+      <c r="C18" s="6"/>
+      <c r="D18" s="6"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A19" s="6"/>
+      <c r="B19" s="6"/>
+      <c r="C19" s="6"/>
+      <c r="D19" s="6"/>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A20" s="6"/>
+      <c r="B20" s="6"/>
+      <c r="C20" s="6"/>
+      <c r="D20" s="6"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>